<commit_message>
fix(template): correct gov form labels + interest rate 7% + fix typo
</commit_message>
<xml_diff>
--- a/estimate-boq-v2/src/assets/templates/boq-master-cgd.xlsx
+++ b/estimate-boq-v2/src/assets/templates/boq-master-cgd.xlsx
@@ -4853,6 +4853,7 @@
     <row r="2">
       <c r="A2" s="373" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -5071,6 +5072,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -5278,6 +5280,7 @@
       <c r="P21" s="537" t="n"/>
       <c r="Q21" s="537" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="377" t="inlineStr">
         <is>
@@ -5404,12 +5407,14 @@
       <c r="AC29" s="21" t="n"/>
       <c r="AD29" s="373" t="n"/>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="B31" s="22" t="n"/>
       <c r="C31" s="22" t="n"/>
       <c r="L31" s="22" t="n"/>
       <c r="M31" s="22" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="B33" s="21" t="n"/>
       <c r="C33" s="21" t="n"/>
@@ -5510,7 +5515,7 @@
       <c r="F1" s="491" t="n"/>
       <c r="G1" s="493" t="inlineStr">
         <is>
-          <t>แบบ ปร.4</t>
+          <t>แบบ ปร.4 (ก)</t>
         </is>
       </c>
       <c r="H1" s="491" t="n"/>
@@ -7095,7 +7100,7 @@
       <c r="H1" s="55" t="n"/>
       <c r="I1" s="27" t="inlineStr">
         <is>
-          <t>แบบ ปร.4</t>
+          <t>แบบ ปร.4 (ก)</t>
         </is>
       </c>
       <c r="K1" s="90" t="n"/>
@@ -20427,31 +20432,31 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A226:E226"/>
+    <mergeCell ref="A138:E138"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A225:E225"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A197:E197"/>
+    <mergeCell ref="A241:E241"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A187:E187"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="A233:E233"/>
+    <mergeCell ref="I5:I6"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A239:E239"/>
-    <mergeCell ref="A226:E226"/>
     <mergeCell ref="A210:E210"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="A138:E138"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A225:E225"/>
     <mergeCell ref="A203:E203"/>
     <mergeCell ref="A219:E219"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A197:E197"/>
-    <mergeCell ref="A241:E241"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A2:I2"/>
     <mergeCell ref="A240:E240"/>
     <mergeCell ref="A209:E209"/>
-    <mergeCell ref="A187:E187"/>
     <mergeCell ref="A165:E165"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A233:E233"/>
-    <mergeCell ref="I5:I6"/>
     <mergeCell ref="C5:C6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -21187,7 +21192,7 @@
       <c r="H1" s="55" t="n"/>
       <c r="J1" s="27" t="inlineStr">
         <is>
-          <t>แบบ ปร.4(ข)</t>
+          <t>แบบ ปร.4 (ข)</t>
         </is>
       </c>
       <c r="K1" s="90" t="n"/>
@@ -22110,7 +22115,7 @@
         </is>
       </c>
       <c r="C16" s="270" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D16" s="673" t="n"/>
       <c r="E16" s="674" t="n"/>
@@ -22385,7 +22390,7 @@
     <col width="9.140625" customWidth="1" style="242" min="264" max="264"/>
     <col width="15.7109375" customWidth="1" style="242" min="265" max="265"/>
     <col width="23.140625" customWidth="1" style="242" min="266" max="266"/>
-    <col hidden="1" style="242" min="267" max="267"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="267" max="267"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="268" max="268"/>
     <col width="9.140625" customWidth="1" style="242" min="269" max="512"/>
     <col width="6" customWidth="1" style="242" min="513" max="513"/>
@@ -22398,7 +22403,7 @@
     <col width="9.140625" customWidth="1" style="242" min="520" max="520"/>
     <col width="15.7109375" customWidth="1" style="242" min="521" max="521"/>
     <col width="23.140625" customWidth="1" style="242" min="522" max="522"/>
-    <col hidden="1" style="242" min="523" max="523"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="523" max="523"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="524" max="524"/>
     <col width="9.140625" customWidth="1" style="242" min="525" max="768"/>
     <col width="6" customWidth="1" style="242" min="769" max="769"/>
@@ -22411,7 +22416,7 @@
     <col width="9.140625" customWidth="1" style="242" min="776" max="776"/>
     <col width="15.7109375" customWidth="1" style="242" min="777" max="777"/>
     <col width="23.140625" customWidth="1" style="242" min="778" max="778"/>
-    <col hidden="1" style="242" min="779" max="779"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="779" max="779"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="780" max="780"/>
     <col width="9.140625" customWidth="1" style="242" min="781" max="1024"/>
     <col width="6" customWidth="1" style="242" min="1025" max="1025"/>
@@ -22424,7 +22429,7 @@
     <col width="9.140625" customWidth="1" style="242" min="1032" max="1032"/>
     <col width="15.7109375" customWidth="1" style="242" min="1033" max="1033"/>
     <col width="23.140625" customWidth="1" style="242" min="1034" max="1034"/>
-    <col hidden="1" style="242" min="1035" max="1035"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="1035" max="1035"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="1036" max="1036"/>
     <col width="9.140625" customWidth="1" style="242" min="1037" max="1280"/>
     <col width="6" customWidth="1" style="242" min="1281" max="1281"/>
@@ -22437,7 +22442,7 @@
     <col width="9.140625" customWidth="1" style="242" min="1288" max="1288"/>
     <col width="15.7109375" customWidth="1" style="242" min="1289" max="1289"/>
     <col width="23.140625" customWidth="1" style="242" min="1290" max="1290"/>
-    <col hidden="1" style="242" min="1291" max="1291"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="1291" max="1291"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="1292" max="1292"/>
     <col width="9.140625" customWidth="1" style="242" min="1293" max="1536"/>
     <col width="6" customWidth="1" style="242" min="1537" max="1537"/>
@@ -22450,7 +22455,7 @@
     <col width="9.140625" customWidth="1" style="242" min="1544" max="1544"/>
     <col width="15.7109375" customWidth="1" style="242" min="1545" max="1545"/>
     <col width="23.140625" customWidth="1" style="242" min="1546" max="1546"/>
-    <col hidden="1" style="242" min="1547" max="1547"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="1547" max="1547"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="1548" max="1548"/>
     <col width="9.140625" customWidth="1" style="242" min="1549" max="1792"/>
     <col width="6" customWidth="1" style="242" min="1793" max="1793"/>
@@ -22463,7 +22468,7 @@
     <col width="9.140625" customWidth="1" style="242" min="1800" max="1800"/>
     <col width="15.7109375" customWidth="1" style="242" min="1801" max="1801"/>
     <col width="23.140625" customWidth="1" style="242" min="1802" max="1802"/>
-    <col hidden="1" style="242" min="1803" max="1803"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="1803" max="1803"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="1804" max="1804"/>
     <col width="9.140625" customWidth="1" style="242" min="1805" max="2048"/>
     <col width="6" customWidth="1" style="242" min="2049" max="2049"/>
@@ -22476,7 +22481,7 @@
     <col width="9.140625" customWidth="1" style="242" min="2056" max="2056"/>
     <col width="15.7109375" customWidth="1" style="242" min="2057" max="2057"/>
     <col width="23.140625" customWidth="1" style="242" min="2058" max="2058"/>
-    <col hidden="1" style="242" min="2059" max="2059"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="2059" max="2059"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="2060" max="2060"/>
     <col width="9.140625" customWidth="1" style="242" min="2061" max="2304"/>
     <col width="6" customWidth="1" style="242" min="2305" max="2305"/>
@@ -22489,7 +22494,7 @@
     <col width="9.140625" customWidth="1" style="242" min="2312" max="2312"/>
     <col width="15.7109375" customWidth="1" style="242" min="2313" max="2313"/>
     <col width="23.140625" customWidth="1" style="242" min="2314" max="2314"/>
-    <col hidden="1" style="242" min="2315" max="2315"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="2315" max="2315"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="2316" max="2316"/>
     <col width="9.140625" customWidth="1" style="242" min="2317" max="2560"/>
     <col width="6" customWidth="1" style="242" min="2561" max="2561"/>
@@ -22502,7 +22507,7 @@
     <col width="9.140625" customWidth="1" style="242" min="2568" max="2568"/>
     <col width="15.7109375" customWidth="1" style="242" min="2569" max="2569"/>
     <col width="23.140625" customWidth="1" style="242" min="2570" max="2570"/>
-    <col hidden="1" style="242" min="2571" max="2571"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="2571" max="2571"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="2572" max="2572"/>
     <col width="9.140625" customWidth="1" style="242" min="2573" max="2816"/>
     <col width="6" customWidth="1" style="242" min="2817" max="2817"/>
@@ -22515,7 +22520,7 @@
     <col width="9.140625" customWidth="1" style="242" min="2824" max="2824"/>
     <col width="15.7109375" customWidth="1" style="242" min="2825" max="2825"/>
     <col width="23.140625" customWidth="1" style="242" min="2826" max="2826"/>
-    <col hidden="1" style="242" min="2827" max="2827"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="2827" max="2827"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="2828" max="2828"/>
     <col width="9.140625" customWidth="1" style="242" min="2829" max="3072"/>
     <col width="6" customWidth="1" style="242" min="3073" max="3073"/>
@@ -22528,7 +22533,7 @@
     <col width="9.140625" customWidth="1" style="242" min="3080" max="3080"/>
     <col width="15.7109375" customWidth="1" style="242" min="3081" max="3081"/>
     <col width="23.140625" customWidth="1" style="242" min="3082" max="3082"/>
-    <col hidden="1" style="242" min="3083" max="3083"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="3083" max="3083"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="3084" max="3084"/>
     <col width="9.140625" customWidth="1" style="242" min="3085" max="3328"/>
     <col width="6" customWidth="1" style="242" min="3329" max="3329"/>
@@ -22541,7 +22546,7 @@
     <col width="9.140625" customWidth="1" style="242" min="3336" max="3336"/>
     <col width="15.7109375" customWidth="1" style="242" min="3337" max="3337"/>
     <col width="23.140625" customWidth="1" style="242" min="3338" max="3338"/>
-    <col hidden="1" style="242" min="3339" max="3339"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="3339" max="3339"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="3340" max="3340"/>
     <col width="9.140625" customWidth="1" style="242" min="3341" max="3584"/>
     <col width="6" customWidth="1" style="242" min="3585" max="3585"/>
@@ -22554,7 +22559,7 @@
     <col width="9.140625" customWidth="1" style="242" min="3592" max="3592"/>
     <col width="15.7109375" customWidth="1" style="242" min="3593" max="3593"/>
     <col width="23.140625" customWidth="1" style="242" min="3594" max="3594"/>
-    <col hidden="1" style="242" min="3595" max="3595"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="3595" max="3595"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="3596" max="3596"/>
     <col width="9.140625" customWidth="1" style="242" min="3597" max="3840"/>
     <col width="6" customWidth="1" style="242" min="3841" max="3841"/>
@@ -22567,7 +22572,7 @@
     <col width="9.140625" customWidth="1" style="242" min="3848" max="3848"/>
     <col width="15.7109375" customWidth="1" style="242" min="3849" max="3849"/>
     <col width="23.140625" customWidth="1" style="242" min="3850" max="3850"/>
-    <col hidden="1" style="242" min="3851" max="3851"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="3851" max="3851"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="3852" max="3852"/>
     <col width="9.140625" customWidth="1" style="242" min="3853" max="4096"/>
     <col width="6" customWidth="1" style="242" min="4097" max="4097"/>
@@ -22580,7 +22585,7 @@
     <col width="9.140625" customWidth="1" style="242" min="4104" max="4104"/>
     <col width="15.7109375" customWidth="1" style="242" min="4105" max="4105"/>
     <col width="23.140625" customWidth="1" style="242" min="4106" max="4106"/>
-    <col hidden="1" style="242" min="4107" max="4107"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="4107" max="4107"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="4108" max="4108"/>
     <col width="9.140625" customWidth="1" style="242" min="4109" max="4352"/>
     <col width="6" customWidth="1" style="242" min="4353" max="4353"/>
@@ -22593,7 +22598,7 @@
     <col width="9.140625" customWidth="1" style="242" min="4360" max="4360"/>
     <col width="15.7109375" customWidth="1" style="242" min="4361" max="4361"/>
     <col width="23.140625" customWidth="1" style="242" min="4362" max="4362"/>
-    <col hidden="1" style="242" min="4363" max="4363"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="4363" max="4363"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="4364" max="4364"/>
     <col width="9.140625" customWidth="1" style="242" min="4365" max="4608"/>
     <col width="6" customWidth="1" style="242" min="4609" max="4609"/>
@@ -22606,7 +22611,7 @@
     <col width="9.140625" customWidth="1" style="242" min="4616" max="4616"/>
     <col width="15.7109375" customWidth="1" style="242" min="4617" max="4617"/>
     <col width="23.140625" customWidth="1" style="242" min="4618" max="4618"/>
-    <col hidden="1" style="242" min="4619" max="4619"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="4619" max="4619"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="4620" max="4620"/>
     <col width="9.140625" customWidth="1" style="242" min="4621" max="4864"/>
     <col width="6" customWidth="1" style="242" min="4865" max="4865"/>
@@ -22619,7 +22624,7 @@
     <col width="9.140625" customWidth="1" style="242" min="4872" max="4872"/>
     <col width="15.7109375" customWidth="1" style="242" min="4873" max="4873"/>
     <col width="23.140625" customWidth="1" style="242" min="4874" max="4874"/>
-    <col hidden="1" style="242" min="4875" max="4875"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="4875" max="4875"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="4876" max="4876"/>
     <col width="9.140625" customWidth="1" style="242" min="4877" max="5120"/>
     <col width="6" customWidth="1" style="242" min="5121" max="5121"/>
@@ -22632,7 +22637,7 @@
     <col width="9.140625" customWidth="1" style="242" min="5128" max="5128"/>
     <col width="15.7109375" customWidth="1" style="242" min="5129" max="5129"/>
     <col width="23.140625" customWidth="1" style="242" min="5130" max="5130"/>
-    <col hidden="1" style="242" min="5131" max="5131"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="5131" max="5131"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="5132" max="5132"/>
     <col width="9.140625" customWidth="1" style="242" min="5133" max="5376"/>
     <col width="6" customWidth="1" style="242" min="5377" max="5377"/>
@@ -22645,7 +22650,7 @@
     <col width="9.140625" customWidth="1" style="242" min="5384" max="5384"/>
     <col width="15.7109375" customWidth="1" style="242" min="5385" max="5385"/>
     <col width="23.140625" customWidth="1" style="242" min="5386" max="5386"/>
-    <col hidden="1" style="242" min="5387" max="5387"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="5387" max="5387"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="5388" max="5388"/>
     <col width="9.140625" customWidth="1" style="242" min="5389" max="5632"/>
     <col width="6" customWidth="1" style="242" min="5633" max="5633"/>
@@ -22658,7 +22663,7 @@
     <col width="9.140625" customWidth="1" style="242" min="5640" max="5640"/>
     <col width="15.7109375" customWidth="1" style="242" min="5641" max="5641"/>
     <col width="23.140625" customWidth="1" style="242" min="5642" max="5642"/>
-    <col hidden="1" style="242" min="5643" max="5643"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="5643" max="5643"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="5644" max="5644"/>
     <col width="9.140625" customWidth="1" style="242" min="5645" max="5888"/>
     <col width="6" customWidth="1" style="242" min="5889" max="5889"/>
@@ -22671,7 +22676,7 @@
     <col width="9.140625" customWidth="1" style="242" min="5896" max="5896"/>
     <col width="15.7109375" customWidth="1" style="242" min="5897" max="5897"/>
     <col width="23.140625" customWidth="1" style="242" min="5898" max="5898"/>
-    <col hidden="1" style="242" min="5899" max="5899"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="5899" max="5899"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="5900" max="5900"/>
     <col width="9.140625" customWidth="1" style="242" min="5901" max="6144"/>
     <col width="6" customWidth="1" style="242" min="6145" max="6145"/>
@@ -22684,7 +22689,7 @@
     <col width="9.140625" customWidth="1" style="242" min="6152" max="6152"/>
     <col width="15.7109375" customWidth="1" style="242" min="6153" max="6153"/>
     <col width="23.140625" customWidth="1" style="242" min="6154" max="6154"/>
-    <col hidden="1" style="242" min="6155" max="6155"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="6155" max="6155"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="6156" max="6156"/>
     <col width="9.140625" customWidth="1" style="242" min="6157" max="6400"/>
     <col width="6" customWidth="1" style="242" min="6401" max="6401"/>
@@ -22697,7 +22702,7 @@
     <col width="9.140625" customWidth="1" style="242" min="6408" max="6408"/>
     <col width="15.7109375" customWidth="1" style="242" min="6409" max="6409"/>
     <col width="23.140625" customWidth="1" style="242" min="6410" max="6410"/>
-    <col hidden="1" style="242" min="6411" max="6411"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="6411" max="6411"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="6412" max="6412"/>
     <col width="9.140625" customWidth="1" style="242" min="6413" max="6656"/>
     <col width="6" customWidth="1" style="242" min="6657" max="6657"/>
@@ -22710,7 +22715,7 @@
     <col width="9.140625" customWidth="1" style="242" min="6664" max="6664"/>
     <col width="15.7109375" customWidth="1" style="242" min="6665" max="6665"/>
     <col width="23.140625" customWidth="1" style="242" min="6666" max="6666"/>
-    <col hidden="1" style="242" min="6667" max="6667"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="6667" max="6667"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="6668" max="6668"/>
     <col width="9.140625" customWidth="1" style="242" min="6669" max="6912"/>
     <col width="6" customWidth="1" style="242" min="6913" max="6913"/>
@@ -22723,7 +22728,7 @@
     <col width="9.140625" customWidth="1" style="242" min="6920" max="6920"/>
     <col width="15.7109375" customWidth="1" style="242" min="6921" max="6921"/>
     <col width="23.140625" customWidth="1" style="242" min="6922" max="6922"/>
-    <col hidden="1" style="242" min="6923" max="6923"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="6923" max="6923"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="6924" max="6924"/>
     <col width="9.140625" customWidth="1" style="242" min="6925" max="7168"/>
     <col width="6" customWidth="1" style="242" min="7169" max="7169"/>
@@ -22736,7 +22741,7 @@
     <col width="9.140625" customWidth="1" style="242" min="7176" max="7176"/>
     <col width="15.7109375" customWidth="1" style="242" min="7177" max="7177"/>
     <col width="23.140625" customWidth="1" style="242" min="7178" max="7178"/>
-    <col hidden="1" style="242" min="7179" max="7179"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="7179" max="7179"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="7180" max="7180"/>
     <col width="9.140625" customWidth="1" style="242" min="7181" max="7424"/>
     <col width="6" customWidth="1" style="242" min="7425" max="7425"/>
@@ -22749,7 +22754,7 @@
     <col width="9.140625" customWidth="1" style="242" min="7432" max="7432"/>
     <col width="15.7109375" customWidth="1" style="242" min="7433" max="7433"/>
     <col width="23.140625" customWidth="1" style="242" min="7434" max="7434"/>
-    <col hidden="1" style="242" min="7435" max="7435"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="7435" max="7435"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="7436" max="7436"/>
     <col width="9.140625" customWidth="1" style="242" min="7437" max="7680"/>
     <col width="6" customWidth="1" style="242" min="7681" max="7681"/>
@@ -22762,7 +22767,7 @@
     <col width="9.140625" customWidth="1" style="242" min="7688" max="7688"/>
     <col width="15.7109375" customWidth="1" style="242" min="7689" max="7689"/>
     <col width="23.140625" customWidth="1" style="242" min="7690" max="7690"/>
-    <col hidden="1" style="242" min="7691" max="7691"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="7691" max="7691"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="7692" max="7692"/>
     <col width="9.140625" customWidth="1" style="242" min="7693" max="7936"/>
     <col width="6" customWidth="1" style="242" min="7937" max="7937"/>
@@ -22775,7 +22780,7 @@
     <col width="9.140625" customWidth="1" style="242" min="7944" max="7944"/>
     <col width="15.7109375" customWidth="1" style="242" min="7945" max="7945"/>
     <col width="23.140625" customWidth="1" style="242" min="7946" max="7946"/>
-    <col hidden="1" style="242" min="7947" max="7947"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="7947" max="7947"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="7948" max="7948"/>
     <col width="9.140625" customWidth="1" style="242" min="7949" max="8192"/>
     <col width="6" customWidth="1" style="242" min="8193" max="8193"/>
@@ -22788,7 +22793,7 @@
     <col width="9.140625" customWidth="1" style="242" min="8200" max="8200"/>
     <col width="15.7109375" customWidth="1" style="242" min="8201" max="8201"/>
     <col width="23.140625" customWidth="1" style="242" min="8202" max="8202"/>
-    <col hidden="1" style="242" min="8203" max="8203"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="8203" max="8203"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="8204" max="8204"/>
     <col width="9.140625" customWidth="1" style="242" min="8205" max="8448"/>
     <col width="6" customWidth="1" style="242" min="8449" max="8449"/>
@@ -22801,7 +22806,7 @@
     <col width="9.140625" customWidth="1" style="242" min="8456" max="8456"/>
     <col width="15.7109375" customWidth="1" style="242" min="8457" max="8457"/>
     <col width="23.140625" customWidth="1" style="242" min="8458" max="8458"/>
-    <col hidden="1" style="242" min="8459" max="8459"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="8459" max="8459"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="8460" max="8460"/>
     <col width="9.140625" customWidth="1" style="242" min="8461" max="8704"/>
     <col width="6" customWidth="1" style="242" min="8705" max="8705"/>
@@ -22814,7 +22819,7 @@
     <col width="9.140625" customWidth="1" style="242" min="8712" max="8712"/>
     <col width="15.7109375" customWidth="1" style="242" min="8713" max="8713"/>
     <col width="23.140625" customWidth="1" style="242" min="8714" max="8714"/>
-    <col hidden="1" style="242" min="8715" max="8715"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="8715" max="8715"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="8716" max="8716"/>
     <col width="9.140625" customWidth="1" style="242" min="8717" max="8960"/>
     <col width="6" customWidth="1" style="242" min="8961" max="8961"/>
@@ -22827,7 +22832,7 @@
     <col width="9.140625" customWidth="1" style="242" min="8968" max="8968"/>
     <col width="15.7109375" customWidth="1" style="242" min="8969" max="8969"/>
     <col width="23.140625" customWidth="1" style="242" min="8970" max="8970"/>
-    <col hidden="1" style="242" min="8971" max="8971"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="8971" max="8971"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="8972" max="8972"/>
     <col width="9.140625" customWidth="1" style="242" min="8973" max="9216"/>
     <col width="6" customWidth="1" style="242" min="9217" max="9217"/>
@@ -22840,7 +22845,7 @@
     <col width="9.140625" customWidth="1" style="242" min="9224" max="9224"/>
     <col width="15.7109375" customWidth="1" style="242" min="9225" max="9225"/>
     <col width="23.140625" customWidth="1" style="242" min="9226" max="9226"/>
-    <col hidden="1" style="242" min="9227" max="9227"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="9227" max="9227"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="9228" max="9228"/>
     <col width="9.140625" customWidth="1" style="242" min="9229" max="9472"/>
     <col width="6" customWidth="1" style="242" min="9473" max="9473"/>
@@ -22853,7 +22858,7 @@
     <col width="9.140625" customWidth="1" style="242" min="9480" max="9480"/>
     <col width="15.7109375" customWidth="1" style="242" min="9481" max="9481"/>
     <col width="23.140625" customWidth="1" style="242" min="9482" max="9482"/>
-    <col hidden="1" style="242" min="9483" max="9483"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="9483" max="9483"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="9484" max="9484"/>
     <col width="9.140625" customWidth="1" style="242" min="9485" max="9728"/>
     <col width="6" customWidth="1" style="242" min="9729" max="9729"/>
@@ -22866,7 +22871,7 @@
     <col width="9.140625" customWidth="1" style="242" min="9736" max="9736"/>
     <col width="15.7109375" customWidth="1" style="242" min="9737" max="9737"/>
     <col width="23.140625" customWidth="1" style="242" min="9738" max="9738"/>
-    <col hidden="1" style="242" min="9739" max="9739"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="9739" max="9739"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="9740" max="9740"/>
     <col width="9.140625" customWidth="1" style="242" min="9741" max="9984"/>
     <col width="6" customWidth="1" style="242" min="9985" max="9985"/>
@@ -22879,7 +22884,7 @@
     <col width="9.140625" customWidth="1" style="242" min="9992" max="9992"/>
     <col width="15.7109375" customWidth="1" style="242" min="9993" max="9993"/>
     <col width="23.140625" customWidth="1" style="242" min="9994" max="9994"/>
-    <col hidden="1" style="242" min="9995" max="9995"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="9995" max="9995"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="9996" max="9996"/>
     <col width="9.140625" customWidth="1" style="242" min="9997" max="10240"/>
     <col width="6" customWidth="1" style="242" min="10241" max="10241"/>
@@ -22892,7 +22897,7 @@
     <col width="9.140625" customWidth="1" style="242" min="10248" max="10248"/>
     <col width="15.7109375" customWidth="1" style="242" min="10249" max="10249"/>
     <col width="23.140625" customWidth="1" style="242" min="10250" max="10250"/>
-    <col hidden="1" style="242" min="10251" max="10251"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="10251" max="10251"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="10252" max="10252"/>
     <col width="9.140625" customWidth="1" style="242" min="10253" max="10496"/>
     <col width="6" customWidth="1" style="242" min="10497" max="10497"/>
@@ -22905,7 +22910,7 @@
     <col width="9.140625" customWidth="1" style="242" min="10504" max="10504"/>
     <col width="15.7109375" customWidth="1" style="242" min="10505" max="10505"/>
     <col width="23.140625" customWidth="1" style="242" min="10506" max="10506"/>
-    <col hidden="1" style="242" min="10507" max="10507"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="10507" max="10507"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="10508" max="10508"/>
     <col width="9.140625" customWidth="1" style="242" min="10509" max="10752"/>
     <col width="6" customWidth="1" style="242" min="10753" max="10753"/>
@@ -22918,7 +22923,7 @@
     <col width="9.140625" customWidth="1" style="242" min="10760" max="10760"/>
     <col width="15.7109375" customWidth="1" style="242" min="10761" max="10761"/>
     <col width="23.140625" customWidth="1" style="242" min="10762" max="10762"/>
-    <col hidden="1" style="242" min="10763" max="10763"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="10763" max="10763"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="10764" max="10764"/>
     <col width="9.140625" customWidth="1" style="242" min="10765" max="11008"/>
     <col width="6" customWidth="1" style="242" min="11009" max="11009"/>
@@ -22931,7 +22936,7 @@
     <col width="9.140625" customWidth="1" style="242" min="11016" max="11016"/>
     <col width="15.7109375" customWidth="1" style="242" min="11017" max="11017"/>
     <col width="23.140625" customWidth="1" style="242" min="11018" max="11018"/>
-    <col hidden="1" style="242" min="11019" max="11019"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="11019" max="11019"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="11020" max="11020"/>
     <col width="9.140625" customWidth="1" style="242" min="11021" max="11264"/>
     <col width="6" customWidth="1" style="242" min="11265" max="11265"/>
@@ -22944,7 +22949,7 @@
     <col width="9.140625" customWidth="1" style="242" min="11272" max="11272"/>
     <col width="15.7109375" customWidth="1" style="242" min="11273" max="11273"/>
     <col width="23.140625" customWidth="1" style="242" min="11274" max="11274"/>
-    <col hidden="1" style="242" min="11275" max="11275"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="11275" max="11275"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="11276" max="11276"/>
     <col width="9.140625" customWidth="1" style="242" min="11277" max="11520"/>
     <col width="6" customWidth="1" style="242" min="11521" max="11521"/>
@@ -22957,7 +22962,7 @@
     <col width="9.140625" customWidth="1" style="242" min="11528" max="11528"/>
     <col width="15.7109375" customWidth="1" style="242" min="11529" max="11529"/>
     <col width="23.140625" customWidth="1" style="242" min="11530" max="11530"/>
-    <col hidden="1" style="242" min="11531" max="11531"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="11531" max="11531"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="11532" max="11532"/>
     <col width="9.140625" customWidth="1" style="242" min="11533" max="11776"/>
     <col width="6" customWidth="1" style="242" min="11777" max="11777"/>
@@ -22970,7 +22975,7 @@
     <col width="9.140625" customWidth="1" style="242" min="11784" max="11784"/>
     <col width="15.7109375" customWidth="1" style="242" min="11785" max="11785"/>
     <col width="23.140625" customWidth="1" style="242" min="11786" max="11786"/>
-    <col hidden="1" style="242" min="11787" max="11787"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="11787" max="11787"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="11788" max="11788"/>
     <col width="9.140625" customWidth="1" style="242" min="11789" max="12032"/>
     <col width="6" customWidth="1" style="242" min="12033" max="12033"/>
@@ -22983,7 +22988,7 @@
     <col width="9.140625" customWidth="1" style="242" min="12040" max="12040"/>
     <col width="15.7109375" customWidth="1" style="242" min="12041" max="12041"/>
     <col width="23.140625" customWidth="1" style="242" min="12042" max="12042"/>
-    <col hidden="1" style="242" min="12043" max="12043"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="12043" max="12043"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="12044" max="12044"/>
     <col width="9.140625" customWidth="1" style="242" min="12045" max="12288"/>
     <col width="6" customWidth="1" style="242" min="12289" max="12289"/>
@@ -22996,7 +23001,7 @@
     <col width="9.140625" customWidth="1" style="242" min="12296" max="12296"/>
     <col width="15.7109375" customWidth="1" style="242" min="12297" max="12297"/>
     <col width="23.140625" customWidth="1" style="242" min="12298" max="12298"/>
-    <col hidden="1" style="242" min="12299" max="12299"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="12299" max="12299"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="12300" max="12300"/>
     <col width="9.140625" customWidth="1" style="242" min="12301" max="12544"/>
     <col width="6" customWidth="1" style="242" min="12545" max="12545"/>
@@ -23009,7 +23014,7 @@
     <col width="9.140625" customWidth="1" style="242" min="12552" max="12552"/>
     <col width="15.7109375" customWidth="1" style="242" min="12553" max="12553"/>
     <col width="23.140625" customWidth="1" style="242" min="12554" max="12554"/>
-    <col hidden="1" style="242" min="12555" max="12555"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="12555" max="12555"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="12556" max="12556"/>
     <col width="9.140625" customWidth="1" style="242" min="12557" max="12800"/>
     <col width="6" customWidth="1" style="242" min="12801" max="12801"/>
@@ -23022,7 +23027,7 @@
     <col width="9.140625" customWidth="1" style="242" min="12808" max="12808"/>
     <col width="15.7109375" customWidth="1" style="242" min="12809" max="12809"/>
     <col width="23.140625" customWidth="1" style="242" min="12810" max="12810"/>
-    <col hidden="1" style="242" min="12811" max="12811"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="12811" max="12811"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="12812" max="12812"/>
     <col width="9.140625" customWidth="1" style="242" min="12813" max="13056"/>
     <col width="6" customWidth="1" style="242" min="13057" max="13057"/>
@@ -23035,7 +23040,7 @@
     <col width="9.140625" customWidth="1" style="242" min="13064" max="13064"/>
     <col width="15.7109375" customWidth="1" style="242" min="13065" max="13065"/>
     <col width="23.140625" customWidth="1" style="242" min="13066" max="13066"/>
-    <col hidden="1" style="242" min="13067" max="13067"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="13067" max="13067"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="13068" max="13068"/>
     <col width="9.140625" customWidth="1" style="242" min="13069" max="13312"/>
     <col width="6" customWidth="1" style="242" min="13313" max="13313"/>
@@ -23048,7 +23053,7 @@
     <col width="9.140625" customWidth="1" style="242" min="13320" max="13320"/>
     <col width="15.7109375" customWidth="1" style="242" min="13321" max="13321"/>
     <col width="23.140625" customWidth="1" style="242" min="13322" max="13322"/>
-    <col hidden="1" style="242" min="13323" max="13323"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="13323" max="13323"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="13324" max="13324"/>
     <col width="9.140625" customWidth="1" style="242" min="13325" max="13568"/>
     <col width="6" customWidth="1" style="242" min="13569" max="13569"/>
@@ -23061,7 +23066,7 @@
     <col width="9.140625" customWidth="1" style="242" min="13576" max="13576"/>
     <col width="15.7109375" customWidth="1" style="242" min="13577" max="13577"/>
     <col width="23.140625" customWidth="1" style="242" min="13578" max="13578"/>
-    <col hidden="1" style="242" min="13579" max="13579"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="13579" max="13579"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="13580" max="13580"/>
     <col width="9.140625" customWidth="1" style="242" min="13581" max="13824"/>
     <col width="6" customWidth="1" style="242" min="13825" max="13825"/>
@@ -23074,7 +23079,7 @@
     <col width="9.140625" customWidth="1" style="242" min="13832" max="13832"/>
     <col width="15.7109375" customWidth="1" style="242" min="13833" max="13833"/>
     <col width="23.140625" customWidth="1" style="242" min="13834" max="13834"/>
-    <col hidden="1" style="242" min="13835" max="13835"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="13835" max="13835"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="13836" max="13836"/>
     <col width="9.140625" customWidth="1" style="242" min="13837" max="14080"/>
     <col width="6" customWidth="1" style="242" min="14081" max="14081"/>
@@ -23087,7 +23092,7 @@
     <col width="9.140625" customWidth="1" style="242" min="14088" max="14088"/>
     <col width="15.7109375" customWidth="1" style="242" min="14089" max="14089"/>
     <col width="23.140625" customWidth="1" style="242" min="14090" max="14090"/>
-    <col hidden="1" style="242" min="14091" max="14091"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="14091" max="14091"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="14092" max="14092"/>
     <col width="9.140625" customWidth="1" style="242" min="14093" max="14336"/>
     <col width="6" customWidth="1" style="242" min="14337" max="14337"/>
@@ -23100,7 +23105,7 @@
     <col width="9.140625" customWidth="1" style="242" min="14344" max="14344"/>
     <col width="15.7109375" customWidth="1" style="242" min="14345" max="14345"/>
     <col width="23.140625" customWidth="1" style="242" min="14346" max="14346"/>
-    <col hidden="1" style="242" min="14347" max="14347"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="14347" max="14347"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="14348" max="14348"/>
     <col width="9.140625" customWidth="1" style="242" min="14349" max="14592"/>
     <col width="6" customWidth="1" style="242" min="14593" max="14593"/>
@@ -23113,7 +23118,7 @@
     <col width="9.140625" customWidth="1" style="242" min="14600" max="14600"/>
     <col width="15.7109375" customWidth="1" style="242" min="14601" max="14601"/>
     <col width="23.140625" customWidth="1" style="242" min="14602" max="14602"/>
-    <col hidden="1" style="242" min="14603" max="14603"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="14603" max="14603"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="14604" max="14604"/>
     <col width="9.140625" customWidth="1" style="242" min="14605" max="14848"/>
     <col width="6" customWidth="1" style="242" min="14849" max="14849"/>
@@ -23126,7 +23131,7 @@
     <col width="9.140625" customWidth="1" style="242" min="14856" max="14856"/>
     <col width="15.7109375" customWidth="1" style="242" min="14857" max="14857"/>
     <col width="23.140625" customWidth="1" style="242" min="14858" max="14858"/>
-    <col hidden="1" style="242" min="14859" max="14859"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="14859" max="14859"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="14860" max="14860"/>
     <col width="9.140625" customWidth="1" style="242" min="14861" max="15104"/>
     <col width="6" customWidth="1" style="242" min="15105" max="15105"/>
@@ -23139,7 +23144,7 @@
     <col width="9.140625" customWidth="1" style="242" min="15112" max="15112"/>
     <col width="15.7109375" customWidth="1" style="242" min="15113" max="15113"/>
     <col width="23.140625" customWidth="1" style="242" min="15114" max="15114"/>
-    <col hidden="1" style="242" min="15115" max="15115"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="15115" max="15115"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="15116" max="15116"/>
     <col width="9.140625" customWidth="1" style="242" min="15117" max="15360"/>
     <col width="6" customWidth="1" style="242" min="15361" max="15361"/>
@@ -23152,7 +23157,7 @@
     <col width="9.140625" customWidth="1" style="242" min="15368" max="15368"/>
     <col width="15.7109375" customWidth="1" style="242" min="15369" max="15369"/>
     <col width="23.140625" customWidth="1" style="242" min="15370" max="15370"/>
-    <col hidden="1" style="242" min="15371" max="15371"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="15371" max="15371"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="15372" max="15372"/>
     <col width="9.140625" customWidth="1" style="242" min="15373" max="15616"/>
     <col width="6" customWidth="1" style="242" min="15617" max="15617"/>
@@ -23165,7 +23170,7 @@
     <col width="9.140625" customWidth="1" style="242" min="15624" max="15624"/>
     <col width="15.7109375" customWidth="1" style="242" min="15625" max="15625"/>
     <col width="23.140625" customWidth="1" style="242" min="15626" max="15626"/>
-    <col hidden="1" style="242" min="15627" max="15627"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="15627" max="15627"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="15628" max="15628"/>
     <col width="9.140625" customWidth="1" style="242" min="15629" max="15872"/>
     <col width="6" customWidth="1" style="242" min="15873" max="15873"/>
@@ -23178,7 +23183,7 @@
     <col width="9.140625" customWidth="1" style="242" min="15880" max="15880"/>
     <col width="15.7109375" customWidth="1" style="242" min="15881" max="15881"/>
     <col width="23.140625" customWidth="1" style="242" min="15882" max="15882"/>
-    <col hidden="1" style="242" min="15883" max="15883"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="15883" max="15883"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="15884" max="15884"/>
     <col width="9.140625" customWidth="1" style="242" min="15885" max="16128"/>
     <col width="6" customWidth="1" style="242" min="16129" max="16129"/>
@@ -23191,7 +23196,7 @@
     <col width="9.140625" customWidth="1" style="242" min="16136" max="16136"/>
     <col width="15.7109375" customWidth="1" style="242" min="16137" max="16137"/>
     <col width="23.140625" customWidth="1" style="242" min="16138" max="16138"/>
-    <col hidden="1" style="242" min="16139" max="16139"/>
+    <col hidden="1" width="13" customWidth="1" style="242" min="16139" max="16139"/>
     <col width="15" bestFit="1" customWidth="1" style="242" min="16140" max="16140"/>
     <col width="9.140625" customWidth="1" style="242" min="16141" max="16384"/>
   </cols>
@@ -23200,7 +23205,7 @@
       <c r="G1" s="207" t="n"/>
       <c r="J1" s="296" t="inlineStr">
         <is>
-          <t>ปร.5 (ช)</t>
+          <t>ปร.5 (ข)</t>
         </is>
       </c>
     </row>
@@ -23684,6 +23689,8 @@
       <c r="H33" s="285" t="n"/>
       <c r="I33" s="285" t="n"/>
     </row>
+    <row r="34"/>
+    <row r="35"/>
     <row r="36" ht="21" customHeight="1">
       <c r="J36" s="88" t="n"/>
     </row>

</xml_diff>